<commit_message>
Status after finalizing 2020 data.
</commit_message>
<xml_diff>
--- a/Data/2020_F013B4_CO_PIT/2020_F013B4_CO_PIT_Management.xlsx
+++ b/Data/2020_F013B4_CO_PIT/2020_F013B4_CO_PIT_Management.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\mnt\Data1\USDA-ALARC\GIS\PDI project\cottondata\Data\2020_F013B4_CO_PIT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F99FCFFE-F0FE-4650-A501-D48F041E9193}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{500AE3FA-68B4-42B5-BD08-F67CB599DDD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16965" yWindow="-21495" windowWidth="17145" windowHeight="19725" tabRatio="756" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-1665" yWindow="-24510" windowWidth="18030" windowHeight="16230" tabRatio="756" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Irrigation" sheetId="4" r:id="rId1"/>
@@ -1230,7 +1230,7 @@
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
-    <numFmt numFmtId="167" formatCode="0.00000"/>
+    <numFmt numFmtId="166" formatCode="0.00000"/>
   </numFmts>
   <fonts count="20" x14ac:knownFonts="1">
     <font>
@@ -1735,7 +1735,7 @@
     <xf numFmtId="0" fontId="1" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1748,9 +1748,8 @@
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -40828,7 +40827,7 @@
         <f>PRODUCT(A7:F7)</f>
         <v>7987500</v>
       </c>
-      <c r="H7" s="12">
+      <c r="H7" s="5">
         <f>G7/G8</f>
         <v>58.387508647834757</v>
       </c>
@@ -41217,7 +41216,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.5703125" bestFit="1" customWidth="1"/>
@@ -41340,7 +41339,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>44158</v>
       </c>
@@ -41348,18 +41347,18 @@
         <v>89</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
       <c r="B18" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>44165</v>
       </c>
@@ -41367,25 +41366,29 @@
         <v>91</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>44169</v>
       </c>
       <c r="B23" t="s">
         <v>92</v>
       </c>
+      <c r="H23">
+        <f>80*0.453592/0.404686*0.45</f>
+        <v>40.350573036873037</v>
+      </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>95</v>
       </c>

</xml_diff>